<commit_message>
Filled ASVS and implement OCC in stock to avoid race conditions
</commit_message>
<xml_diff>
--- a/Deliverables/Sprint_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Sprint_1/ASVS_5.0_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\Documents\GitHub\desofs2026-tue_crr_3\Documentation\Reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\Documents\GitHub\desofs2026-tue_crr_3\Deliverables\Sprint_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0786169B-60A6-41A0-9BA4-6C7C0537F973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8656B3-B0BD-48D3-A8AC-C22E265C62C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2087" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2125" uniqueCount="959">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2828,6 +2828,120 @@
   </si>
   <si>
     <t>Email address, postal addressare assigned a protection level that determines encryption on  logging.</t>
+  </si>
+  <si>
+    <t>Inputs is processed directly by strongly typed .NET models .Direct String inputs used for file names (`ReportName`) are canonicalized immediately upon receipt in `SanitizeFileName` by stripping directory separators and traversal sequences , and resolving to a safe filename using `Path.GetFileName`before operating on it</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L235</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L258</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Database: The repository layer uses Entity Framework Core parameterized LINQ queries, delegating parameter escaping to the database provider itself.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Output escaping is performed as a final step during serialization via "EscapeCsvField", which escapes spreadsheet formula triggers and prevents CSV/Formula injection.</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Infrastructure/Persistence/Repositories/TeaRepository.cs#L8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">he application does not manually construct JSON strings via concatenation.  API serialization is handled  by  .NET </t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Presentation/OrderController.cs#L11</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Infrastructure/Persistence/Repositories/OrderRepository.cs#L10</t>
+  </si>
+  <si>
+    <t>Repositories interact with the database through Entity Framework Core.This uses parameterized queries, ensuring that variables are sent as SQL parameters rather than concatenated SQL strings</t>
+  </si>
+  <si>
+    <t>Data passed to external interpreters or potentially risky contexts is parameterized or escaped beforehand. Relational database queries use EF Core parameterization, while CSV exports utilize the method `EscapeCsvField`</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Infrastructure/Persistence/Repositories/SessionRepository.cs</t>
+  </si>
+  <si>
+    <t>The application does not dynamically evaluate or compile format string templates using untrusted inputs. All string formatting throughout the codebase (such as in filename generation and CSV writing) relies on compile-time string interpolation ($) or hardcoded format strings</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L205</t>
+  </si>
+  <si>
+    <t>The application is built entirely in managed C#  which is a memory-safe language. There is no use of unsafe blocks or manual pointers</t>
+  </si>
+  <si>
+    <t>Input range validations are applied to numeric inputs (such as quantities and prices). Furthermore, financial calculations utilize the .NET 'decimal' data type, which natively throws an `OverflowException`</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderDTOs.cs#L7</t>
+  </si>
+  <si>
+    <t>Standard memory allocation is managed by the .NET Garbage Collector. Unmanaged system resources, such as stream writers and memory streams, are wrapped in standard 'using' statements ensuring guaranteed resource release immediately after use</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L212</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The application deserializes incoming API payloads strictly into defined, strongly typed C# DTOs using 'System.Text.Json'. It does not accept or deserialize arbitrary  types  and the use of of insecure serializers  is prohibited</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Presentation/OrderController.cs#L119</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The application utilizes positive validation (allow-listing). Incoming data is validated against strictly defined schemas and  strict numeric ranges </t>
+  </si>
+  <si>
+    <t>Validation rules are strictly enforced at the trusted server-side Application Service layer</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L190</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Combinations of related data items are validated for logical consistency on the server. For example, in sales report generation, the system validates that `StartDate` is chronologically earlier than or equal to `EndDate` before executing the database query</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L197</t>
+  </si>
+  <si>
+    <t>State transitions are validated sequentially in the domain layer. For example, an order cannot be transitioned to a 'Canceled' state unless its current sequential state permits it</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Domain/Orders/Order.cs#L42</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Logical business boundaries are strictly enforced. Standard users can only retrieve or cancel orders that match their authenticated  userId.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The application utilizes the Unit of Work pattern to coordinate persistence across repositories. Business transactions are kept in-memory and committed atomically. </t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Domain/Orders/Order.cs#L39</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Application/Orders/OrderService.cs#L38</t>
+  </si>
+  <si>
+    <t>The application implements standard anti-automation and resource protection controls using the built-in ASP.NET Core Rate Limiting middleware. This prevents automated scripts from triggering denial of service (DoS), resource exhaustion, or data scraping.</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Infrastructure/Security/RateLimiting.cs#L7</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/ff5dce5c732d9649d8f6ac4460f32af19f100fe6/TeaShop/TeaShop/Presentation/AuthController.cs#L28</t>
+  </si>
+  <si>
+    <t>The application prevents race conditions and over-allocation  using Optimistic Concurrency Control (OCC)</t>
+  </si>
+  <si>
+    <t>Fill after commit</t>
   </si>
 </sst>
 </file>
@@ -3301,10 +3415,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -3485,10 +3599,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.42105263157894735</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.7142857142857143</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -3669,7 +3783,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -3850,10 +3964,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.36666666666666664</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.61538461538461542</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4519,41 +4633,41 @@
       </c>
       <c r="D6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,1)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" s="5">
         <f t="shared" ref="E6:E20" si="0">IF(C6=0,"",D6/C6)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F6" s="4">
         <v>19</v>
       </c>
       <c r="G6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,2)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H6" s="5">
         <f t="shared" ref="H6:H22" si="1">IF(F6=0,"",G6/F6)</f>
-        <v>0</v>
+        <v>0.42105263157894735</v>
       </c>
       <c r="I6" s="4">
         <v>3</v>
       </c>
       <c r="J6" s="4">
         <f>COUNTIFS('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant",'V1 - Encoding and Sanitization'!$E$2:$E$36,3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="5">
         <f t="shared" ref="K6:K13" si="2">IF(I6=0,"",J6/I6)</f>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="L6" s="4">
         <f>COUNTIF('V1 - Encoding and Sanitization'!$F$2:$F$36,"Compliant")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" ref="M6:M22" si="3">IF(B6=0,"",L6/B6)</f>
-        <v>0</v>
+        <v>0.36666666666666664</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -4568,22 +4682,22 @@
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant",'V2 - Validation and Business Lo'!$E$2:$E$18,1)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="F7" s="7">
         <v>7</v>
       </c>
       <c r="G7" s="7">
         <f>COUNTIFS('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant",'V2 - Validation and Business Lo'!$E$2:$E$18,2)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H7" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="I7" s="7">
         <v>2</v>
@@ -4598,11 +4712,11 @@
       </c>
       <c r="L7" s="7">
         <f>COUNTIF('V2 - Validation and Business Lo'!$F$2:$F$18,"Compliant")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M7" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.61538461538461542</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -5348,11 +5462,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>8.7606837606837601E-2</v>
+        <v>0.15427350427350428</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5360,11 +5474,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>2.4000509294626941E-2</v>
+        <v>9.0785117874901164E-2</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5372,19 +5486,19 @@
       </c>
       <c r="J23" s="10">
         <f>SUM(J6:J22)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="11">
         <f>IFERROR(AVERAGE(K6:K22),"")</f>
-        <v>0</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>3.2645606265591778E-2</v>
+        <v>9.0413328739196608E-2</v>
       </c>
     </row>
   </sheetData>
@@ -10227,10 +10341,14 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>921</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>922</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
@@ -10249,10 +10367,14 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>925</v>
+      </c>
+      <c r="H4" s="25" t="s">
+        <v>927</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
@@ -10285,7 +10407,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
@@ -10307,7 +10429,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G7" s="21"/>
       <c r="H7" s="21"/>
@@ -10329,10 +10451,14 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>928</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>929</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
@@ -10351,10 +10477,14 @@
         <v>1</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>931</v>
+      </c>
+      <c r="H9" s="25" t="s">
+        <v>930</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
@@ -10373,7 +10503,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
@@ -10395,7 +10525,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21"/>
@@ -10417,7 +10547,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
@@ -10439,7 +10569,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="21"/>
@@ -10461,7 +10591,7 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
@@ -10483,10 +10613,14 @@
         <v>3</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>926</v>
+      </c>
+      <c r="H15" s="25" t="s">
+        <v>923</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
@@ -10519,7 +10653,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
@@ -10541,7 +10675,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
@@ -10563,10 +10697,14 @@
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G19" s="16" t="s">
+        <v>932</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>933</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
@@ -10585,7 +10723,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
@@ -10607,7 +10745,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
@@ -10629,7 +10767,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
@@ -10651,7 +10789,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
@@ -10673,7 +10811,7 @@
         <v>2</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
@@ -10695,7 +10833,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
@@ -10717,10 +10855,14 @@
         <v>2</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G26" s="21" t="s">
+        <v>934</v>
+      </c>
+      <c r="H26" s="21" t="s">
+        <v>935</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
@@ -10739,7 +10881,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
@@ -10761,7 +10903,7 @@
         <v>3</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G28" s="21"/>
       <c r="H28" s="21"/>
@@ -10797,9 +10939,11 @@
         <v>2</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G30" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>936</v>
+      </c>
       <c r="H30" s="16"/>
     </row>
     <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -10819,10 +10963,14 @@
         <v>2</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>937</v>
+      </c>
+      <c r="H31" s="25" t="s">
+        <v>938</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
@@ -10841,10 +10989,14 @@
         <v>2</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>939</v>
+      </c>
+      <c r="H32" s="24" t="s">
+        <v>940</v>
+      </c>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="13" t="s">
@@ -10877,7 +11029,7 @@
         <v>1</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
@@ -10899,10 +11051,14 @@
         <v>2</v>
       </c>
       <c r="F35" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G35" s="21" t="s">
+        <v>941</v>
+      </c>
+      <c r="H35" s="21" t="s">
+        <v>942</v>
+      </c>
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="14" t="s">
@@ -10921,7 +11077,7 @@
         <v>3</v>
       </c>
       <c r="F36" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
@@ -10944,6 +11100,16 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H3" r:id="rId1" location="L235" xr:uid="{A84892FB-9B9D-4523-9A7E-2DA48FCFCA1F}"/>
+    <hyperlink ref="H4" r:id="rId2" location="L8" xr:uid="{BCA6D288-8A4B-4A20-854D-994C10E48932}"/>
+    <hyperlink ref="H15" r:id="rId3" location="L258" xr:uid="{25DD70A4-00A4-4831-9049-70628FB5F38C}"/>
+    <hyperlink ref="H8" r:id="rId4" location="L11" xr:uid="{3B438980-FE39-4E81-B42B-2CC167323DC9}"/>
+    <hyperlink ref="H9" r:id="rId5" location="L10" xr:uid="{08CC7360-7339-4631-994D-0EB25FEAA689}"/>
+    <hyperlink ref="H32" r:id="rId6" location="L212" xr:uid="{E5DAB9EF-00BE-4435-A7C3-C2D3D103CCF6}"/>
+    <hyperlink ref="H19" r:id="rId7" xr:uid="{EA877C8B-DE1F-48BC-A5DF-EFCEF855CB16}"/>
+    <hyperlink ref="H31" r:id="rId8" location="L7" xr:uid="{79E4D5CA-BA87-4EF3-A1E7-91EA186E8A66}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -10951,7 +11117,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -11101,10 +11267,14 @@
         <v>1</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>943</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>938</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
@@ -11123,10 +11293,14 @@
         <v>1</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>944</v>
+      </c>
+      <c r="H8" s="25" t="s">
+        <v>945</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
@@ -11145,10 +11319,14 @@
         <v>2</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>946</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>947</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
@@ -11181,10 +11359,14 @@
         <v>1</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>948</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>949</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
@@ -11203,10 +11385,14 @@
         <v>2</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>950</v>
+      </c>
+      <c r="H12" s="25" t="s">
+        <v>952</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
@@ -11225,10 +11411,14 @@
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>951</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>953</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
@@ -11247,10 +11437,14 @@
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>957</v>
+      </c>
+      <c r="H14" s="21" t="s">
+        <v>958</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
@@ -11269,7 +11463,7 @@
         <v>3</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -11288,7 +11482,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
     </row>
-    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>140</v>
       </c>
@@ -11305,12 +11499,19 @@
         <v>2</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-    </row>
-    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>954</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>955</v>
+      </c>
+      <c r="I17" s="27" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
         <v>140</v>
       </c>
@@ -11327,7 +11528,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>45</v>
+        <v>924</v>
       </c>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
@@ -11350,6 +11551,15 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H8" r:id="rId1" location="L190" xr:uid="{598CAFA4-055B-4A86-9723-2701E48D6B5E}"/>
+    <hyperlink ref="H9" r:id="rId2" location="L197" xr:uid="{E7854916-D85D-4CE1-863D-0D2D57C64538}"/>
+    <hyperlink ref="H11" r:id="rId3" location="L42" xr:uid="{3FAE36F8-A7C4-4842-87C8-EDB25C1DDC8E}"/>
+    <hyperlink ref="H12" r:id="rId4" location="L39" xr:uid="{3EDD0CD1-7836-4B5E-A687-06AD31F95DBF}"/>
+    <hyperlink ref="H13" r:id="rId5" location="L38" xr:uid="{A91F97D6-FD86-4237-AEBD-473B19266593}"/>
+    <hyperlink ref="H17" r:id="rId6" location="L7" xr:uid="{D773793C-1794-4A22-8B98-45097F9F4EC2}"/>
+    <hyperlink ref="I17" r:id="rId7" location="L28" xr:uid="{937F3CFB-6A68-4930-B95F-B6AE300E54FD}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
ASVS V6.1 authentication documentation
</commit_message>
<xml_diff>
--- a/Deliverables/Sprint_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Sprint_1/ASVS_5.0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85DB334-B03A-4C87-B5F6-2A37DF57900E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294FFC32-95D0-4FCC-986F-38B5C4A50360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="770" yWindow="740" windowWidth="14400" windowHeight="7270" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2131" uniqueCount="965">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="969">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2960,6 +2960,18 @@
   </si>
   <si>
     <t>Requirements.md - NFR-01, NFR-02, NFR-05, Section 3 (BR-01 to BR-06)</t>
+  </si>
+  <si>
+    <t>Authentication protection controls are documented, including rate limiting requirements for sensitive endpoints such as login and registration.</t>
+  </si>
+  <si>
+    <t>Requirements.md - NFR-8</t>
+  </si>
+  <si>
+    <t>A context-specific password policy is documented. It defines that commonly used passwords and application-specific terms must not be accepted during registration or password change operations.</t>
+  </si>
+  <si>
+    <t>Requirements.md - BR-07 Password Policy</t>
   </si>
 </sst>
 </file>
@@ -3448,7 +3460,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.23076923076923078</c:v>
+                  <c:v>0.30769230769230771</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.5</c:v>
@@ -3632,7 +3644,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.18181818181818182</c:v>
+                  <c:v>0.22727272727272727</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>8.3333333333333329E-2</c:v>
@@ -3997,7 +4009,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.14893617021276595</c:v>
+                  <c:v>0.19148936170212766</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.21052631578947367</c:v>
@@ -4896,22 +4908,22 @@
       </c>
       <c r="D11" s="7">
         <f>COUNTIFS('V6 - Authentication'!$F$2:$F$56,"Compliant",'V6 - Authentication'!$E$2:$E$56,1)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" s="8">
         <f t="shared" si="0"/>
-        <v>0.23076923076923078</v>
+        <v>0.30769230769230771</v>
       </c>
       <c r="F11" s="7">
         <v>22</v>
       </c>
       <c r="G11" s="7">
         <f>COUNTIFS('V6 - Authentication'!$F$2:$F$56,"Compliant",'V6 - Authentication'!$E$2:$E$56,2)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11" s="8">
         <f t="shared" si="1"/>
-        <v>0.18181818181818182</v>
+        <v>0.22727272727272727</v>
       </c>
       <c r="I11" s="7">
         <v>12</v>
@@ -4926,11 +4938,11 @@
       </c>
       <c r="L11" s="7">
         <f>COUNTIF('V6 - Authentication'!$F$2:$F$56,"Compliant")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M11" s="8">
         <f t="shared" si="3"/>
-        <v>0.14893617021276595</v>
+        <v>0.19148936170212766</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -5480,11 +5492,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0.17094017094017094</v>
+        <v>0.17606837606837605</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5492,11 +5504,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0.10759184056397678</v>
+        <v>0.11026563735542062</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -5512,11 +5524,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.10398798937268075</v>
+        <v>0.10649111828381967</v>
       </c>
     </row>
   </sheetData>
@@ -13389,10 +13401,14 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>965</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>966</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
@@ -13411,10 +13427,14 @@
         <v>2</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>967</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>968</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">

</xml_diff>

<commit_message>
Updated ASVS V6.2 password security compliance evaluation
</commit_message>
<xml_diff>
--- a/Deliverables/Sprint_1/ASVS_5.0_Tracker.xlsx
+++ b/Deliverables/Sprint_1/ASVS_5.0_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\OneDrive\Ambiente de Trabalho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294FFC32-95D0-4FCC-986F-38B5C4A50360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888F67A8-43FA-4AE3-AF46-CF961B15182B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="770" yWindow="740" windowWidth="14400" windowHeight="7270" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="500" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="969">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2139" uniqueCount="972">
   <si>
     <t>OWASP ASVS 5.0 – Compliance Tracker</t>
   </si>
@@ -2972,6 +2972,15 @@
   </si>
   <si>
     <t>Requirements.md - BR-07 Password Policy</t>
+  </si>
+  <si>
+    <t>Passwords are validated against compromised password databases using Have I Been Pwned integration and are also checked against application-specific forbidden terms.</t>
+  </si>
+  <si>
+    <t>The application enforces password length and blacklist validation but does not restrict the character composition of passwords.</t>
+  </si>
+  <si>
+    <t>https://github.com/mei-desofs/desofs2026-tue_crr_3/blob/8eac90d29c53f3f94c5afe7d0e70417f54ea3fd0/TeaShop/TeaShop/Presentation/AuthController.cs</t>
   </si>
 </sst>
 </file>
@@ -3460,7 +3469,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.30769230769230771</c:v>
+                  <c:v>0.46153846153846156</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.5</c:v>
@@ -4009,7 +4018,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.19148936170212766</c:v>
+                  <c:v>0.23404255319148937</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.21052631578947367</c:v>
@@ -4908,11 +4917,11 @@
       </c>
       <c r="D11" s="7">
         <f>COUNTIFS('V6 - Authentication'!$F$2:$F$56,"Compliant",'V6 - Authentication'!$E$2:$E$56,1)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E11" s="8">
         <f t="shared" si="0"/>
-        <v>0.30769230769230771</v>
+        <v>0.46153846153846156</v>
       </c>
       <c r="F11" s="7">
         <v>22</v>
@@ -4938,11 +4947,11 @@
       </c>
       <c r="L11" s="7">
         <f>COUNTIF('V6 - Authentication'!$F$2:$F$56,"Compliant")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M11" s="8">
         <f t="shared" si="3"/>
-        <v>0.19148936170212766</v>
+        <v>0.23404255319148937</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -5492,11 +5501,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0.17606837606837605</v>
+        <v>0.18632478632478636</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -5524,11 +5533,11 @@
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.10649111828381967</v>
+        <v>0.10899424719495861</v>
       </c>
     </row>
   </sheetData>
@@ -13546,7 +13555,7 @@
       <c r="G9" s="16" t="s">
         <v>904</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="24" t="s">
         <v>897</v>
       </c>
     </row>
@@ -13567,10 +13576,14 @@
         <v>1</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
+        <v>892</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>969</v>
+      </c>
+      <c r="H10" s="25" t="s">
+        <v>971</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14" t="s">
@@ -13589,10 +13602,14 @@
         <v>1</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
+        <v>892</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>970</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>971</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
@@ -14571,6 +14588,9 @@
     <hyperlink ref="H7" r:id="rId1" location="L21" xr:uid="{F596CCA9-524A-46C7-9C77-F6EA6F450E91}"/>
     <hyperlink ref="H8" r:id="rId2" location="L52" xr:uid="{65E8B584-A00F-4884-A727-264FF99EB138}"/>
     <hyperlink ref="H18" r:id="rId3" location="L27" xr:uid="{E112FC84-77A3-41FD-92F9-0CF4A1D171BE}"/>
+    <hyperlink ref="H9" r:id="rId4" location="L117" xr:uid="{91645EE2-7393-4503-92C1-CC7EA3162839}"/>
+    <hyperlink ref="H10" r:id="rId5" xr:uid="{C370F1BE-887F-4566-9C70-1B36A846657C}"/>
+    <hyperlink ref="H11" r:id="rId6" xr:uid="{2001B137-FFE0-4FB0-88EE-DCDC3C42F888}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>